<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table07-08
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table07.xlsx
+++ b/sources/table_normalization/xlsx/economy-table07.xlsx
@@ -198,12 +198,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="4"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <name val="Arial Unicode MS"/>
@@ -254,10 +248,17 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
       <sz val="4"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="5">
@@ -319,7 +320,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -349,39 +350,39 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -406,14 +407,15 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Заголовок 1" xfId="1" builtinId="16"/>
@@ -923,7 +925,7 @@
   <cols>
     <col min="1" max="2" width="7.7265625" customWidth="1"/>
     <col min="3" max="3" width="12.26953125" customWidth="1"/>
-    <col min="4" max="4" width="2.7265625" customWidth="1"/>
+    <col min="4" max="4" width="4.26953125" customWidth="1"/>
     <col min="5" max="5" width="14.1796875" customWidth="1"/>
     <col min="6" max="6" width="2.7265625" customWidth="1"/>
     <col min="7" max="7" width="14.7265625" customWidth="1"/>
@@ -1022,28 +1024,28 @@
       <c r="B6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="36" t="s">
+      <c r="F6" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="35" t="s">
+      <c r="G6" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="35" t="s">
+      <c r="I6" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="38" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2392,18 +2394,18 @@
       </c>
     </row>
     <row r="49" spans="1:10" ht="15" customHeight="1">
-      <c r="A49" s="38" t="s">
+      <c r="A49" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="B49" s="39"/>
-      <c r="C49" s="40"/>
-      <c r="D49" s="41"/>
-      <c r="E49" s="40"/>
-      <c r="F49" s="41"/>
-      <c r="G49" s="40"/>
-      <c r="H49" s="41"/>
-      <c r="I49" s="40"/>
-      <c r="J49" s="41"/>
+      <c r="B49" s="40"/>
+      <c r="C49" s="37"/>
+      <c r="D49" s="37"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="37"/>
+      <c r="H49" s="37"/>
+      <c r="I49" s="37"/>
+      <c r="J49" s="37"/>
     </row>
     <row r="50" spans="1:10" ht="15" customHeight="1">
       <c r="A50" s="15" t="s">
@@ -2594,9 +2596,9 @@
     <hyperlink ref="A2:B2" location="Contents!A1" display="Back to contents"/>
   </hyperlinks>
   <pageMargins left="0.196850393700787" right="0.196850393700787" top="0.196850393700787" bottom="0.196850393700787" header="0.39370078740157499" footer="0.39370078740157499"/>
-  <pageSetup paperSize="9" scale="76" orientation="portrait" horizontalDpi="300"/>
+  <pageSetup paperSize="9" scale="76" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>